<commit_message>
adjust upload excel data
</commit_message>
<xml_diff>
--- a/trial_upload.xlsx
+++ b/trial_upload.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Works\THE RESONANZ\CODING\_WEBSITE\_TRIAL\reservation-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B76AF671-C1EC-40CE-AA82-68CDE56AE74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DF671F-B249-4DD7-9EBA-E272C30C9FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14580" yWindow="5730" windowWidth="21600" windowHeight="12645" xr2:uid="{EA4D115C-2700-43A2-8523-F08C559A643E}"/>
+    <workbookView xWindow="7125" yWindow="3465" windowWidth="21600" windowHeight="12645" xr2:uid="{EA4D115C-2700-43A2-8523-F08C559A643E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>name</t>
   </si>
@@ -106,6 +106,42 @@
   </si>
   <si>
     <t>X342</t>
+  </si>
+  <si>
+    <t>company</t>
+  </si>
+  <si>
+    <t>position</t>
+  </si>
+  <si>
+    <t>PT AB</t>
+  </si>
+  <si>
+    <t>PT NE</t>
+  </si>
+  <si>
+    <t>PT BO</t>
+  </si>
+  <si>
+    <t>PT CH</t>
+  </si>
+  <si>
+    <t>PT TI</t>
+  </si>
+  <si>
+    <t>CEO</t>
+  </si>
+  <si>
+    <t>CFO</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Technician</t>
+  </si>
+  <si>
+    <t>HRD</t>
   </si>
 </sst>
 </file>
@@ -469,106 +505,144 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27BC3E3D-1D19-4878-8B7C-DDE0DF180096}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{142F8AEC-FC7C-444F-BD4A-679999924D8F}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{F159A207-42E8-4E26-A7F0-337CA0EA1B99}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{2702CF60-5E3B-4F6A-8354-0DD829941F7F}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{7437A277-7BF0-4462-AF1B-907033301D42}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{717E6326-AF15-44B8-84AB-01C028E7DF06}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{142F8AEC-FC7C-444F-BD4A-679999924D8F}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{F159A207-42E8-4E26-A7F0-337CA0EA1B99}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{2702CF60-5E3B-4F6A-8354-0DD829941F7F}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{7437A277-7BF0-4462-AF1B-907033301D42}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{717E6326-AF15-44B8-84AB-01C028E7DF06}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add date and time to upload
</commit_message>
<xml_diff>
--- a/trial_upload.xlsx
+++ b/trial_upload.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Works\THE RESONANZ\CODING\_WEBSITE\_TRIAL\reservation-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DF671F-B249-4DD7-9EBA-E272C30C9FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A3A8B3-02F7-43FD-BBB4-0B8BC4802F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7125" yWindow="3465" windowWidth="21600" windowHeight="12645" xr2:uid="{EA4D115C-2700-43A2-8523-F08C559A643E}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{EA4D115C-2700-43A2-8523-F08C559A643E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>name</t>
   </si>
@@ -142,6 +142,18 @@
   </si>
   <si>
     <t>HRD</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>15:00</t>
   </si>
 </sst>
 </file>
@@ -505,7 +517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27BC3E3D-1D19-4878-8B7C-DDE0DF180096}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -514,9 +526,11 @@
     <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -535,8 +549,14 @@
       <c r="F1" t="s">
         <v>3</v>
       </c>
+      <c r="G1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -555,8 +575,14 @@
       <c r="F2" t="s">
         <v>19</v>
       </c>
+      <c r="G2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -575,8 +601,14 @@
       <c r="F3" t="s">
         <v>20</v>
       </c>
+      <c r="G3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -595,8 +627,14 @@
       <c r="F4" t="s">
         <v>21</v>
       </c>
+      <c r="G4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -615,8 +653,14 @@
       <c r="F5" t="s">
         <v>22</v>
       </c>
+      <c r="G5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -634,6 +678,12 @@
       </c>
       <c r="F6" t="s">
         <v>23</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>